<commit_message>
Updated database + added simulation settings + updated PBL code
</commit_message>
<xml_diff>
--- a/data_ProjectTemplate/GridNodes_ProjectTemplate.xlsx
+++ b/data_ProjectTemplate/GridNodes_ProjectTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AteHe\Desktop\Modellen\Zero_ProjectTemplate\data_ProjectTemplate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bas\Desktop\Github\LUX_ProjectTemplate\data_ProjectTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DEB889D-2041-4F2C-A25F-DF09BC321324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A45FF97-E959-485F-A39E-20CE894A73CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{A7529885-FB18-401C-977B-A3275EF3AD02}"/>
+    <workbookView xWindow="73125" yWindow="4005" windowWidth="23235" windowHeight="11235" xr2:uid="{A7529885-FB18-401C-977B-A3275EF3AD02}"/>
   </bookViews>
   <sheets>
     <sheet name="gridnodes" sheetId="2" r:id="rId1"/>
@@ -836,21 +836,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7BCE184-E6B7-4248-9F1F-EFB645AF205B}">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultColWidth="18.7265625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="18.77734375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.81640625" customWidth="1"/>
+    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.77734375" customWidth="1"/>
+    <col min="12" max="12" width="21.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
@@ -888,7 +889,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>18</v>
       </c>

</xml_diff>